<commit_message>
update excel sprint 2
</commit_message>
<xml_diff>
--- a/Sprints/SOEN 341 MasterChef agile planning.xlsx
+++ b/Sprints/SOEN 341 MasterChef agile planning.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="210">
   <si>
     <t>Master Chef</t>
   </si>
@@ -403,7 +403,7 @@
     <t>17thFebruary</t>
   </si>
   <si>
-    <t>US.04</t>
+    <t>#4</t>
   </si>
   <si>
     <t>Story 4: Create, Edit, and Delete Recipes
@@ -516,6 +516,140 @@
   </si>
   <si>
     <t>Build Create Recipe UI form, Build Edit Recipe UI form, Build Delete Recipe UI confirmation, Frontend validation for recipe forms, Create unit tests — Recipe CRUD</t>
+  </si>
+  <si>
+    <t>#5</t>
+  </si>
+  <si>
+    <t>Story 5: Search Recipes
+ As a user, I want to search for recipes by keyword so that I can quickly find relevant meals from the recipe collection.</t>
+  </si>
+  <si>
+    <t>Implement Search Recipe API</t>
+  </si>
+  <si>
+    <t>Develop GET /api/recipes/search?q= endpoint. Perform case-insensitive text search on recipe title, description, and ingredients fields. Return paginated results.</t>
+  </si>
+  <si>
+    <t>25th February</t>
+  </si>
+  <si>
+    <t>Search query performance depends on proper indexing; needs testing with larger datasets.</t>
+  </si>
+  <si>
+    <t>Create recipe database schema (US.04)</t>
+  </si>
+  <si>
+    <t>Add database index for search fields</t>
+  </si>
+  <si>
+    <t>Add text indexes (or equivalent) on the title, description, and ingredients fields to ensure search queries perform efficiently.</t>
+  </si>
+  <si>
+    <t>26th February</t>
+  </si>
+  <si>
+    <t>Without indexing, search degrades significantly at scale; must be done before integration tests.</t>
+  </si>
+  <si>
+    <t>Nicolas</t>
+  </si>
+  <si>
+    <t>Build Search UI component</t>
+  </si>
+  <si>
+    <t>Add a search bar to the recipes page that triggers the search API on input with debouncing. Display matching results in a list/grid. Show 'No results found' state.</t>
+  </si>
+  <si>
+    <t>Self-contained UI component; low coupling to other sprint stories.</t>
+  </si>
+  <si>
+    <t>Create unit tests — Search</t>
+  </si>
+  <si>
+    <t>Write unit tests for search endpoint: keyword match, case-insensitivity, empty query, no-results scenario, and pagination.</t>
+  </si>
+  <si>
+    <t>Well-defined inputs and outputs; straightforward to test.</t>
+  </si>
+  <si>
+    <t>Integration testing — Search</t>
+  </si>
+  <si>
+    <t>Seed the database with sample recipes and test the full search flow from UI input to rendered results. Verify debouncing and empty-state handling.</t>
+  </si>
+  <si>
+    <t>Requires seed data; otherwise low risk.</t>
+  </si>
+  <si>
+    <t>Build Search UI component, Implement Search Recipe API, Add database index for search fields, Create unit tests — Search</t>
+  </si>
+  <si>
+    <t>US.06</t>
+  </si>
+  <si>
+    <t>Story 6: Filter Recipes
+ As a user, I want to filter the recipe list by time, difficulty, cost, and dietary tags so that I can find meals that fit my constraints and preferences.</t>
+  </si>
+  <si>
+    <t>Implement Filter Recipe API</t>
+  </si>
+  <si>
+    <t>Extend GET /api/recipes to accept query parameters: max_time, difficulty, dietary_tags (comma-separated). Apply filters server-side and return matching recipes.</t>
+  </si>
+  <si>
+    <t>Multiple filter combinations must all work correctly; edge cases (no results, combined filters) need coverage.</t>
+  </si>
+  <si>
+    <t>Create recipe database schema (US.04), Implement Create Recipe API (US.04)</t>
+  </si>
+  <si>
+    <t>Build Filter UI panel</t>
+  </si>
+  <si>
+    <t>Add a collapsible filter panel to the recipes page with controls for: time range slider, difficulty dropdown, and dietary tag checkboxes (matching profile preferences).</t>
+  </si>
+  <si>
+    <t>Multiple interactive controls; state management for combined filters is moderately complex.</t>
+  </si>
+  <si>
+    <t>Build Search UI component (US.05)</t>
+  </si>
+  <si>
+    <t>Navnit, Joey</t>
+  </si>
+  <si>
+    <t>Combine search and filter</t>
+  </si>
+  <si>
+    <t>Ensure search and filter parameters can be applied simultaneously in a single API call. Update the frontend to pass both search query and active filters together.</t>
+  </si>
+  <si>
+    <t>Integration point between two features; parameter merging logic must be tested carefully.</t>
+  </si>
+  <si>
+    <t>Implement Search Recipe API (US.05), Implement Filter Recipe API</t>
+  </si>
+  <si>
+    <t>Create unit tests — Filter</t>
+  </si>
+  <si>
+    <t>Write unit tests for filter endpoint: each filter type individually, combined filters, no-match scenario, and invalid parameter handling.</t>
+  </si>
+  <si>
+    <t>Well-scoped test suite; low risk of external dependencies.</t>
+  </si>
+  <si>
+    <t>Integration testing — Filter</t>
+  </si>
+  <si>
+    <t>Seed the database with diverse recipe data and test all filter combinations from the UI through to the rendered results. Verify combined search + filter works correctly.</t>
+  </si>
+  <si>
+    <t>Combined search+filter path is the highest-risk integration scenario.</t>
+  </si>
+  <si>
+    <t>Build Filter UI panel, Implement Filter Recipe API, Combine search and filter, Create unit tests — Filter</t>
   </si>
 </sst>
 </file>
@@ -644,7 +778,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="39">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -721,13 +855,13 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" textRotation="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" textRotation="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" textRotation="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" textRotation="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" textRotation="0" vertical="top" wrapText="1"/>
@@ -743,6 +877,24 @@
     </xf>
     <xf borderId="1" fillId="8" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" textRotation="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="7" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="8" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3438,7 +3590,7 @@
       </c>
     </row>
     <row r="14" ht="40.5" customHeight="1">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="19" t="s">
         <v>128</v>
       </c>
       <c r="B14" s="23"/>
@@ -3485,18 +3637,18 @@
       <c r="Y14" s="1"/>
       <c r="Z14" s="1"/>
     </row>
-    <row r="15">
-      <c r="A15" s="25" t="s">
+    <row r="15" ht="38.25" customHeight="1">
+      <c r="A15" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="B15" s="26"/>
-      <c r="C15" s="27" t="s">
+      <c r="B15" s="25"/>
+      <c r="C15" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="D15" s="27" t="s">
+      <c r="D15" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="27">
         <v>2.0</v>
       </c>
       <c r="F15" s="18" t="s">
@@ -3508,10 +3660,10 @@
       <c r="H15" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="I15" s="27" t="s">
+      <c r="I15" s="26" t="s">
         <v>140</v>
       </c>
-      <c r="J15" s="27" t="s">
+      <c r="J15" s="26" t="s">
         <v>135</v>
       </c>
       <c r="K15" s="13" t="s">
@@ -3534,17 +3686,17 @@
       <c r="Z15" s="30"/>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="s">
+      <c r="A16" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="27" t="s">
+      <c r="B16" s="25"/>
+      <c r="C16" s="26" t="s">
         <v>141</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="D16" s="26" t="s">
         <v>142</v>
       </c>
-      <c r="E16" s="25">
+      <c r="E16" s="27">
         <v>1.0</v>
       </c>
       <c r="F16" s="18" t="s">
@@ -3556,10 +3708,10 @@
       <c r="H16" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="I16" s="27" t="s">
+      <c r="I16" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="J16" s="27" t="s">
+      <c r="J16" s="26" t="s">
         <v>138</v>
       </c>
       <c r="K16" s="13" t="s">
@@ -3582,20 +3734,20 @@
       <c r="Z16" s="30"/>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="27" t="s">
+      <c r="B17" s="25"/>
+      <c r="C17" s="26" t="s">
         <v>144</v>
       </c>
-      <c r="D17" s="27" t="s">
+      <c r="D17" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="E17" s="25">
+      <c r="E17" s="27">
         <v>3.0</v>
       </c>
-      <c r="F17" s="25" t="s">
+      <c r="F17" s="27" t="s">
         <v>146</v>
       </c>
       <c r="G17" s="28" t="s">
@@ -3604,13 +3756,13 @@
       <c r="H17" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="I17" s="27" t="s">
+      <c r="I17" s="26" t="s">
         <v>147</v>
       </c>
-      <c r="J17" s="27" t="s">
+      <c r="J17" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="K17" s="25" t="s">
+      <c r="K17" s="27" t="s">
         <v>75</v>
       </c>
       <c r="L17" s="30"/>
@@ -3630,20 +3782,20 @@
       <c r="Z17" s="30"/>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="B18" s="26"/>
-      <c r="C18" s="27" t="s">
+      <c r="B18" s="25"/>
+      <c r="C18" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="D18" s="27" t="s">
+      <c r="D18" s="26" t="s">
         <v>149</v>
       </c>
-      <c r="E18" s="25">
+      <c r="E18" s="27">
         <v>2.0</v>
       </c>
-      <c r="F18" s="25" t="s">
+      <c r="F18" s="27" t="s">
         <v>122</v>
       </c>
       <c r="G18" s="28" t="s">
@@ -3652,13 +3804,13 @@
       <c r="H18" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="I18" s="27" t="s">
+      <c r="I18" s="26" t="s">
         <v>150</v>
       </c>
-      <c r="J18" s="27" t="s">
+      <c r="J18" s="26" t="s">
         <v>151</v>
       </c>
-      <c r="K18" s="25" t="s">
+      <c r="K18" s="27" t="s">
         <v>68</v>
       </c>
       <c r="L18" s="30"/>
@@ -3678,20 +3830,20 @@
       <c r="Z18" s="30"/>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="27" t="s">
+      <c r="B19" s="25"/>
+      <c r="C19" s="26" t="s">
         <v>152</v>
       </c>
-      <c r="D19" s="27" t="s">
+      <c r="D19" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="E19" s="25">
+      <c r="E19" s="27">
         <v>1.0</v>
       </c>
-      <c r="F19" s="25" t="s">
+      <c r="F19" s="27" t="s">
         <v>122</v>
       </c>
       <c r="G19" s="32" t="s">
@@ -3700,13 +3852,13 @@
       <c r="H19" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="I19" s="27" t="s">
+      <c r="I19" s="26" t="s">
         <v>154</v>
       </c>
-      <c r="J19" s="27" t="s">
+      <c r="J19" s="26" t="s">
         <v>155</v>
       </c>
-      <c r="K19" s="25" t="s">
+      <c r="K19" s="27" t="s">
         <v>68</v>
       </c>
       <c r="L19" s="30"/>
@@ -3726,20 +3878,20 @@
       <c r="Z19" s="30"/>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="B20" s="26"/>
-      <c r="C20" s="27" t="s">
+      <c r="B20" s="25"/>
+      <c r="C20" s="26" t="s">
         <v>156</v>
       </c>
-      <c r="D20" s="27" t="s">
+      <c r="D20" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="E20" s="25">
+      <c r="E20" s="27">
         <v>1.0</v>
       </c>
-      <c r="F20" s="25" t="s">
+      <c r="F20" s="27" t="s">
         <v>146</v>
       </c>
       <c r="G20" s="32" t="s">
@@ -3748,13 +3900,13 @@
       <c r="H20" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="I20" s="27" t="s">
+      <c r="I20" s="26" t="s">
         <v>158</v>
       </c>
-      <c r="J20" s="27" t="s">
+      <c r="J20" s="26" t="s">
         <v>144</v>
       </c>
-      <c r="K20" s="25" t="s">
+      <c r="K20" s="27" t="s">
         <v>75</v>
       </c>
       <c r="L20" s="30"/>
@@ -3774,20 +3926,20 @@
       <c r="Z20" s="30"/>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="27" t="s">
+      <c r="B21" s="25"/>
+      <c r="C21" s="26" t="s">
         <v>159</v>
       </c>
-      <c r="D21" s="27" t="s">
+      <c r="D21" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="E21" s="25">
+      <c r="E21" s="27">
         <v>2.0</v>
       </c>
-      <c r="F21" s="25" t="s">
+      <c r="F21" s="27" t="s">
         <v>122</v>
       </c>
       <c r="G21" s="32" t="s">
@@ -3796,10 +3948,10 @@
       <c r="H21" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="I21" s="27" t="s">
+      <c r="I21" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="J21" s="27" t="s">
+      <c r="J21" s="26" t="s">
         <v>161</v>
       </c>
       <c r="K21" s="13" t="s">
@@ -3822,20 +3974,20 @@
       <c r="Z21" s="30"/>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="s">
+      <c r="A22" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="B22" s="26"/>
-      <c r="C22" s="27" t="s">
+      <c r="B22" s="25"/>
+      <c r="C22" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="D22" s="27" t="s">
+      <c r="D22" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="E22" s="25">
+      <c r="E22" s="27">
         <v>2.0</v>
       </c>
-      <c r="F22" s="25" t="s">
+      <c r="F22" s="27" t="s">
         <v>122</v>
       </c>
       <c r="G22" s="28" t="s">
@@ -3844,10 +3996,10 @@
       <c r="H22" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="I22" s="27" t="s">
+      <c r="I22" s="26" t="s">
         <v>164</v>
       </c>
-      <c r="J22" s="27" t="s">
+      <c r="J22" s="26" t="s">
         <v>165</v>
       </c>
       <c r="K22" s="13" t="s">
@@ -3870,17 +4022,489 @@
       <c r="Z22" s="30"/>
     </row>
     <row r="23">
-      <c r="K23" s="13"/>
-    </row>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
+      <c r="A23" s="33" t="s">
+        <v>166</v>
+      </c>
+      <c r="B23" s="34" t="s">
+        <v>167</v>
+      </c>
+      <c r="C23" s="35" t="s">
+        <v>168</v>
+      </c>
+      <c r="D23" s="35" t="s">
+        <v>169</v>
+      </c>
+      <c r="E23" s="33">
+        <v>2.0</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="G23" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="H23" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="I23" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="J23" s="35" t="s">
+        <v>172</v>
+      </c>
+      <c r="K23" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1"/>
+      <c r="R23" s="1"/>
+      <c r="S23" s="1"/>
+      <c r="T23" s="1"/>
+      <c r="U23" s="1"/>
+      <c r="V23" s="1"/>
+      <c r="W23" s="1"/>
+      <c r="X23" s="1"/>
+      <c r="Y23" s="1"/>
+      <c r="Z23" s="1"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="33" t="s">
+        <v>166</v>
+      </c>
+      <c r="B24" s="23"/>
+      <c r="C24" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="E24" s="18">
+        <v>1.0</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="G24" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="H24" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="I24" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="J24" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="K24" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1"/>
+      <c r="R24" s="1"/>
+      <c r="S24" s="1"/>
+      <c r="T24" s="1"/>
+      <c r="U24" s="1"/>
+      <c r="V24" s="1"/>
+      <c r="W24" s="1"/>
+      <c r="X24" s="1"/>
+      <c r="Y24" s="1"/>
+      <c r="Z24" s="1"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="33" t="s">
+        <v>166</v>
+      </c>
+      <c r="B25" s="23"/>
+      <c r="C25" s="17" t="s">
+        <v>178</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="E25" s="18">
+        <v>2.0</v>
+      </c>
+      <c r="F25" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="G25" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="H25" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="I25" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="J25" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="K25" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1"/>
+      <c r="R25" s="1"/>
+      <c r="S25" s="1"/>
+      <c r="T25" s="1"/>
+      <c r="U25" s="1"/>
+      <c r="V25" s="1"/>
+      <c r="W25" s="1"/>
+      <c r="X25" s="1"/>
+      <c r="Y25" s="1"/>
+      <c r="Z25" s="1"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="33" t="s">
+        <v>166</v>
+      </c>
+      <c r="B26" s="23"/>
+      <c r="C26" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="E26" s="18">
+        <v>1.0</v>
+      </c>
+      <c r="F26" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="G26" s="38" t="s">
+        <v>26</v>
+      </c>
+      <c r="H26" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="I26" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="J26" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="K26" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
+      <c r="R26" s="1"/>
+      <c r="S26" s="1"/>
+      <c r="T26" s="1"/>
+      <c r="U26" s="1"/>
+      <c r="V26" s="1"/>
+      <c r="W26" s="1"/>
+      <c r="X26" s="1"/>
+      <c r="Y26" s="1"/>
+      <c r="Z26" s="1"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="33" t="s">
+        <v>166</v>
+      </c>
+      <c r="B27" s="23"/>
+      <c r="C27" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="E27" s="18">
+        <v>1.0</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="G27" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="H27" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="I27" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="J27" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="K27" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1"/>
+      <c r="R27" s="1"/>
+      <c r="S27" s="1"/>
+      <c r="T27" s="1"/>
+      <c r="U27" s="1"/>
+      <c r="V27" s="1"/>
+      <c r="W27" s="1"/>
+      <c r="X27" s="1"/>
+      <c r="Y27" s="1"/>
+      <c r="Z27" s="1"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="B28" s="34" t="s">
+        <v>189</v>
+      </c>
+      <c r="C28" s="35" t="s">
+        <v>190</v>
+      </c>
+      <c r="D28" s="35" t="s">
+        <v>191</v>
+      </c>
+      <c r="E28" s="33">
+        <v>2.0</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="G28" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="H28" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="I28" s="35" t="s">
+        <v>192</v>
+      </c>
+      <c r="J28" s="35" t="s">
+        <v>193</v>
+      </c>
+      <c r="K28" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1"/>
+      <c r="R28" s="1"/>
+      <c r="S28" s="1"/>
+      <c r="T28" s="1"/>
+      <c r="U28" s="1"/>
+      <c r="V28" s="1"/>
+      <c r="W28" s="1"/>
+      <c r="X28" s="1"/>
+      <c r="Y28" s="1"/>
+      <c r="Z28" s="1"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="B29" s="23"/>
+      <c r="C29" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="E29" s="18">
+        <v>3.0</v>
+      </c>
+      <c r="F29" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="G29" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="H29" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="I29" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="J29" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="K29" s="18" t="s">
+        <v>198</v>
+      </c>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1"/>
+      <c r="R29" s="1"/>
+      <c r="S29" s="1"/>
+      <c r="T29" s="1"/>
+      <c r="U29" s="1"/>
+      <c r="V29" s="1"/>
+      <c r="W29" s="1"/>
+      <c r="X29" s="1"/>
+      <c r="Y29" s="1"/>
+      <c r="Z29" s="1"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="B30" s="23"/>
+      <c r="C30" s="17" t="s">
+        <v>199</v>
+      </c>
+      <c r="D30" s="17" t="s">
+        <v>200</v>
+      </c>
+      <c r="E30" s="18">
+        <v>2.0</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="G30" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="H30" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="I30" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="J30" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="K30" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1"/>
+      <c r="R30" s="1"/>
+      <c r="S30" s="1"/>
+      <c r="T30" s="1"/>
+      <c r="U30" s="1"/>
+      <c r="V30" s="1"/>
+      <c r="W30" s="1"/>
+      <c r="X30" s="1"/>
+      <c r="Y30" s="1"/>
+      <c r="Z30" s="1"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="B31" s="23"/>
+      <c r="C31" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="E31" s="18">
+        <v>2.0</v>
+      </c>
+      <c r="F31" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="G31" s="38" t="s">
+        <v>26</v>
+      </c>
+      <c r="H31" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="I31" s="17" t="s">
+        <v>205</v>
+      </c>
+      <c r="J31" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="K31" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1"/>
+      <c r="R31" s="1"/>
+      <c r="S31" s="1"/>
+      <c r="T31" s="1"/>
+      <c r="U31" s="1"/>
+      <c r="V31" s="1"/>
+      <c r="W31" s="1"/>
+      <c r="X31" s="1"/>
+      <c r="Y31" s="1"/>
+      <c r="Z31" s="1"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="B32" s="23"/>
+      <c r="C32" s="17" t="s">
+        <v>206</v>
+      </c>
+      <c r="D32" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="E32" s="18">
+        <v>2.0</v>
+      </c>
+      <c r="F32" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="G32" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="H32" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="I32" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="J32" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="K32" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+      <c r="Q32" s="1"/>
+      <c r="R32" s="1"/>
+      <c r="S32" s="1"/>
+      <c r="T32" s="1"/>
+      <c r="U32" s="1"/>
+      <c r="V32" s="1"/>
+      <c r="W32" s="1"/>
+      <c r="X32" s="1"/>
+      <c r="Y32" s="1"/>
+      <c r="Z32" s="1"/>
+    </row>
     <row r="33"/>
     <row r="34"/>
     <row r="35"/>

</xml_diff>